<commit_message>
Changed to Non Headless
</commit_message>
<xml_diff>
--- a/reports/ExcelReport/ExtentExcel.xlsx
+++ b/reports/ExcelReport/ExtentExcel.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="64">
   <si>
     <t>Duration</t>
   </si>
@@ -189,46 +189,46 @@
     <t>device</t>
   </si>
   <si>
-    <t>Mar 18, 2026 1:00:38 am</t>
+    <t>Jul 01, 2026 3:26:20 PM</t>
   </si>
   <si>
-    <t>Mar 18, 2026 1:00:02 am</t>
+    <t>Jul 01, 2026 3:26:09 PM</t>
   </si>
   <si>
-    <t>Mar 18, 2026 1:00:37 am</t>
+    <t>Jul 01, 2026 3:26:18 PM</t>
   </si>
   <si>
-    <t>35.756 s</t>
+    <t>9.032 s</t>
   </si>
   <si>
     <t>100%</t>
   </si>
   <si>
-    <t>Login Data Driven from Excel</t>
+    <t>Login with valid credentials</t>
   </si>
   <si>
-    <t>33.677 s</t>
+    <t>6.318 s</t>
   </si>
   <si>
     <t>Login</t>
   </si>
   <si>
-    <t>33.756 s</t>
+    <t>Successful user registration</t>
   </si>
   <si>
-    <t>13.506 s</t>
+    <t>7.392 s</t>
   </si>
   <si>
-    <t>33.760 s</t>
+    <t>User Registration</t>
   </si>
   <si>
-    <t>33.634 s</t>
+    <t>@sanity</t>
   </si>
   <si>
-    <t>@datadriven</t>
+    <t>6.323 s</t>
   </si>
   <si>
-    <t>33.809 s</t>
+    <t>7.393 s</t>
   </si>
 </sst>
 </file>
@@ -1796,46 +1796,28 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Scenarios!$B$22:$B$26</c:f>
+              <c:f>Scenarios!$B$22:$B$23</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Login Data Driven from Excel</c:v>
+                  <c:v>Login with valid credentials</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Login Data Driven from Excel</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Login Data Driven from Excel</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Login Data Driven from Excel</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Login Data Driven from Excel</c:v>
+                  <c:v>Successful user registration</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scenarios!$H$22:$H$26</c:f>
+              <c:f>Scenarios!$H$22:$H$23</c:f>
               <c:numCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>4.0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>4.0</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>4.0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4.0</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4.0</c:v>
+                  <c:v>5.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1892,30 +1874,21 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Scenarios!$B$22:$B$26</c:f>
+              <c:f>Scenarios!$B$22:$B$23</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Login Data Driven from Excel</c:v>
+                  <c:v>Login with valid credentials</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Login Data Driven from Excel</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Login Data Driven from Excel</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Login Data Driven from Excel</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Login Data Driven from Excel</c:v>
+                  <c:v>Successful user registration</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scenarios!$J$22:$J$26</c:f>
+              <c:f>Scenarios!$J$22:$J$23</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -1971,30 +1944,21 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Scenarios!$B$22:$B$26</c:f>
+              <c:f>Scenarios!$B$22:$B$23</c:f>
               <c:strCache>
-                <c:ptCount val="5"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>Login Data Driven from Excel</c:v>
+                  <c:v>Login with valid credentials</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Login Data Driven from Excel</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>Login Data Driven from Excel</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>Login Data Driven from Excel</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>Login Data Driven from Excel</c:v>
+                  <c:v>Successful user registration</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Scenarios!$I$22:$I$26</c:f>
+              <c:f>Scenarios!$I$22:$I$23</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -2394,7 +2358,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>@datadriven</c:v>
+                  <c:v>@sanity</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2405,7 +2369,7 @@
               <c:numCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>5.0</c:v>
+                  <c:v>2.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2467,7 +2431,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>@datadriven</c:v>
+                  <c:v>@sanity</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2535,7 +2499,7 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>@datadriven</c:v>
+                  <c:v>@sanity</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2747,22 +2711,28 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Features!$B$22</c:f>
+              <c:f>Features!$B$22:$B$23</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>Login</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>User Registration</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Features!$F$22</c:f>
+              <c:f>Features!$F$22:$F$23</c:f>
               <c:numCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>5.0</c:v>
+                  <c:v>1.0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2819,18 +2789,21 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Features!$B$22</c:f>
+              <c:f>Features!$B$22:$B$23</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>Login</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>User Registration</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Features!$H$22</c:f>
+              <c:f>Features!$H$22:$H$23</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -2886,18 +2859,21 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Features!$B$22</c:f>
+              <c:f>Features!$B$22:$B$23</c:f>
               <c:strCache>
-                <c:ptCount val="1"/>
+                <c:ptCount val="2"/>
                 <c:pt idx="0">
                   <c:v>Login</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>User Registration</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Features!$G$22</c:f>
+              <c:f>Features!$G$22:$G$23</c:f>
               <c:numCache/>
             </c:numRef>
           </c:val>
@@ -5830,7 +5806,7 @@
     <col min="7" max="7" customWidth="true" width="20.85546875"/>
   </cols>
   <sheetData/>
-  <sheetProtection sheet="true" password="F4BF" scenarios="true" objects="true"/>
+  <sheetProtection sheet="true" password="B699" scenarios="true" objects="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -5839,7 +5815,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B20:J26"/>
+  <dimension ref="B20:J23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="1.42578125"/>
@@ -5924,103 +5900,28 @@
     </row>
     <row r="23">
       <c r="B23" s="54" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C23" s="55" t="s">
         <v>29</v>
       </c>
       <c r="D23" s="56" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E23" s="54" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F23" s="55" t="s">
         <v>29</v>
       </c>
       <c r="G23" s="57" t="n">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="H23" s="58" t="n">
-        <v>4.0</v>
+        <v>5.0</v>
       </c>
       <c r="I23" s="59"/>
       <c r="J23" s="60"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="54" t="s">
-        <v>55</v>
-      </c>
-      <c r="C24" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D24" s="56" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" s="54" t="s">
-        <v>57</v>
-      </c>
-      <c r="F24" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G24" s="57" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="H24" s="58" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="I24" s="59"/>
-      <c r="J24" s="60"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="54" t="s">
-        <v>55</v>
-      </c>
-      <c r="C25" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D25" s="56" t="s">
-        <v>60</v>
-      </c>
-      <c r="E25" s="54" t="s">
-        <v>57</v>
-      </c>
-      <c r="F25" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G25" s="57" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="H25" s="58" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="I25" s="59"/>
-      <c r="J25" s="60"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="54" t="s">
-        <v>55</v>
-      </c>
-      <c r="C26" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" s="56" t="s">
-        <v>61</v>
-      </c>
-      <c r="E26" s="54" t="s">
-        <v>57</v>
-      </c>
-      <c r="F26" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="G26" s="57" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="H26" s="58" t="n">
-        <v>4.0</v>
-      </c>
-      <c r="I26" s="59"/>
-      <c r="J26" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6036,7 +5937,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B20:I31"/>
+  <dimension ref="B20:I28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="1.28515625"/>
@@ -6078,13 +5979,13 @@
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s" s="54">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C22" s="57" t="n">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="D22" s="58" t="n">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="E22" s="59"/>
       <c r="F22" s="60"/>
@@ -6112,7 +6013,7 @@
     </row>
     <row r="27">
       <c r="B27" s="54" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C27" s="62" t="s">
         <v>57</v>
@@ -6130,67 +6031,28 @@
     </row>
     <row r="28">
       <c r="B28" s="53"/>
-      <c r="C28" s="53"/>
+      <c r="C28" s="62" t="s">
+        <v>60</v>
+      </c>
       <c r="D28" s="53"/>
       <c r="E28" s="53"/>
       <c r="F28" s="53"/>
       <c r="G28" s="53"/>
       <c r="H28" s="62" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="I28" s="55" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="53"/>
-      <c r="C29" s="53"/>
-      <c r="D29" s="53"/>
-      <c r="E29" s="53"/>
-      <c r="F29" s="53"/>
-      <c r="G29" s="53"/>
-      <c r="H29" s="62" t="s">
-        <v>55</v>
-      </c>
-      <c r="I29" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="53"/>
-      <c r="C30" s="53"/>
-      <c r="D30" s="53"/>
-      <c r="E30" s="53"/>
-      <c r="F30" s="53"/>
-      <c r="G30" s="53"/>
-      <c r="H30" s="62" t="s">
-        <v>55</v>
-      </c>
-      <c r="I30" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="53"/>
-      <c r="C31" s="53"/>
-      <c r="D31" s="53"/>
-      <c r="E31" s="53"/>
-      <c r="F31" s="53"/>
-      <c r="G31" s="53"/>
-      <c r="H31" s="62" t="s">
-        <v>55</v>
-      </c>
-      <c r="I31" s="55" t="s">
-        <v>29</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B20:B21"/>
     <mergeCell ref="C20:G20"/>
     <mergeCell ref="C26:G26"/>
-    <mergeCell ref="B27:B31"/>
-    <mergeCell ref="C27:G31"/>
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="C28:G28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6200,7 +6062,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B18:M22"/>
+  <dimension ref="B18:M23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="2.0"/>
@@ -6281,13 +6143,13 @@
         <v>29</v>
       </c>
       <c r="D22" s="56" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E22" s="57" t="n">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
       <c r="F22" s="58" t="n">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
       <c r="G22" s="59"/>
       <c r="H22" s="60"/>
@@ -6295,13 +6157,43 @@
         <v>54</v>
       </c>
       <c r="J22" s="57" t="n">
-        <v>20.0</v>
+        <v>4.0</v>
       </c>
       <c r="K22" s="58" t="n">
-        <v>20.0</v>
+        <v>4.0</v>
       </c>
       <c r="L22" s="59"/>
       <c r="M22" s="60"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="54" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="55" t="s">
+        <v>29</v>
+      </c>
+      <c r="D23" s="56" t="s">
+        <v>63</v>
+      </c>
+      <c r="E23" s="57" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="F23" s="58" t="n">
+        <v>1.0</v>
+      </c>
+      <c r="G23" s="59"/>
+      <c r="H23" s="60"/>
+      <c r="I23" s="61" t="s">
+        <v>54</v>
+      </c>
+      <c r="J23" s="57" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="K23" s="58" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="L23" s="59"/>
+      <c r="M23" s="60"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -6360,19 +6252,19 @@
         <v>3</v>
       </c>
       <c r="D2" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>9</v>
       </c>
       <c r="F2" t="n" s="0">
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="G2" t="s" s="0">
         <v>12</v>
       </c>
       <c r="H2" t="n" s="0">
-        <v>20.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -6427,21 +6319,21 @@
       </c>
       <c r="D5" t="n" s="0">
         <f>SUM(D2:D4)</f>
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>20</v>
       </c>
       <c r="F5" t="n" s="0">
         <f>SUM(F2:F4)</f>
-        <v>5.0</v>
+        <v>2.0</v>
       </c>
       <c r="G5" t="s" s="0">
         <v>21</v>
       </c>
       <c r="H5" t="n" s="0">
         <f>SUM(H2:H4)</f>
-        <v>20.0</v>
+        <v>9.0</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>